<commit_message>
Add new Excel files for durian and vegetable recommendations, and update existing files with new data.
</commit_message>
<xml_diff>
--- a/files/durian-recommendations.xlsx
+++ b/files/durian-recommendations.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jusep\Desktop\PROJECTS\amia-microsite.github.io\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C9B8DF1-13F0-4F8C-B16F-55DD402AD444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E8CFF1-42DE-4E24-AEB7-6744F25B73E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E2D1DC89-D079-3B4D-864B-8CE149E3E279}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{E2D1DC89-D079-3B4D-864B-8CE149E3E279}"/>
   </bookViews>
   <sheets>
     <sheet name="Durian_10Day(Municipal)" sheetId="9" r:id="rId1"/>
     <sheet name="Durian_10Day_SMS" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="Durian_Seasonal(Provincial)" sheetId="13" r:id="rId3"/>
-    <sheet name="Guidelines" sheetId="14" r:id="rId4"/>
-    <sheet name="Durian_(General)" sheetId="6" state="hidden" r:id="rId5"/>
-    <sheet name="Durian_SMS" sheetId="3" state="hidden" r:id="rId6"/>
-    <sheet name="Durian_Special" sheetId="10" state="hidden" r:id="rId7"/>
-    <sheet name="Durian_Special_SMS" sheetId="12" state="hidden" r:id="rId8"/>
+    <sheet name="Guidelines" sheetId="16" r:id="rId4"/>
+    <sheet name="References" sheetId="17" r:id="rId5"/>
+    <sheet name="Durian_(General)" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="Durian_SMS" sheetId="3" state="hidden" r:id="rId7"/>
+    <sheet name="Durian_Special" sheetId="10" state="hidden" r:id="rId8"/>
+    <sheet name="Durian_Special_SMS" sheetId="12" state="hidden" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="114">
   <si>
     <t>Crop Stage</t>
   </si>
@@ -270,15 +271,558 @@
   </si>
   <si>
     <t>Maturing Stage</t>
+  </si>
+  <si>
+    <t>CROP STAGES</t>
+  </si>
+  <si>
+    <t>FARMING ACTIVITIES</t>
+  </si>
+  <si>
+    <t>Harvesting, Post Harvest Management</t>
+  </si>
+  <si>
+    <t>10-DAY WEATHER FORECAST</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>Definition</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ten(10) consecutive days with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">light rains </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">or Five(5) consecutive days with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>no rain</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Three(3) consecutive days with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">moderate rains </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">or Two(2) consecutive days with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>heavy rains</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rainfall conditions are balanced</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and do not meet the threshold for water stress or flooding hazards during the 10-day forecast period</t>
+    </r>
+  </si>
+  <si>
+    <t>SEASONAL FORECAST</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Two(2) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">below normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(21% - 60% reduction from average) rainfall conditions</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Three(3) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">below normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(21% - 60% reduction from average) rainfall conditions;
+Two(2) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">way below normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(more than 60% reduction from average) rainfall conditions</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Three(3) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>way</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">below normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(&gt;60% reduction from average);
+Five(5) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">below normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(21% - 60% reduction from average) rainfall condition</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Two(2) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>above normal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (21% - 60% from average)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Three(3) or more consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">above normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(&gt;60% increase from average);
+Two(2) consecutive months of </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">way above normal </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(more than 60% increase from average)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rainfall conditions are near normal</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, without sustained anomalies of below normal or above normal rainfall</t>
+    </r>
+  </si>
+  <si>
+    <t>Land Preparation, Transplanting</t>
+  </si>
+  <si>
+    <t>Water Management, Nutrient Management</t>
+  </si>
+  <si>
+    <t>Pest Management, Nutrient Management</t>
+  </si>
+  <si>
+    <t>IMPACT OUTLOOK AND MANAGEMENT RECOMMENDATION GUIDELINES</t>
+  </si>
+  <si>
+    <t>1. Provide recommendations for every farm activity listed under each climate risk.</t>
+  </si>
+  <si>
+    <t>- All Impact Outlook and Management Recommendation fields must be completed, and no cell should be left blank</t>
+  </si>
+  <si>
+    <t>- Each farm activity must have at least one management recommendation tailored to the specific climate condition and corresponding impact outlook.</t>
+  </si>
+  <si>
+    <t>- Multiple recommendations may be provided if necessary</t>
+  </si>
+  <si>
+    <r>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>x.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If the farm activity is nursery establishment under water shortage risk, provide recommendations such as improved moisture conservation techniques.</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Ensure alignment between climate risk, impact outlook, and recommendation.</t>
+  </si>
+  <si>
+    <t>- Impact outlooks must directly relate to the specified climate risk and include both negative and positive effects where applicable</t>
+  </si>
+  <si>
+    <t>- Recommendations must directly respond to the stated impacts</t>
+  </si>
+  <si>
+    <r>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>x.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If flooding risk may cause soil erosion, recommend elevated nursery beds or drainage construction.</t>
+    </r>
+  </si>
+  <si>
+    <t>3. Provide detailed, practical, and farmer-level applicable management recommendations.</t>
+  </si>
+  <si>
+    <t>- Avoid vague instructions unless paired with a clear and actionable measure</t>
+  </si>
+  <si>
+    <r>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>x.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Instead of “monitor plants,” use “monitor plants for pest infestation and apply neem extract if early pest signs are observed.”</t>
+    </r>
+  </si>
+  <si>
+    <t>5. Climate risks are standardized and fixed. Do not add, remove, or modify the provided climate risk categories.</t>
+  </si>
+  <si>
+    <t>6. Include crop insurance (PCIC) recommendations where appropriate, particularly during vulnerable crop stages such as flowering or fruiting.</t>
+  </si>
+  <si>
+    <r>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>x.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Recommend PCIC crop insurance enrollment during reproductive and maturing stages for high-value crops.</t>
+    </r>
+  </si>
+  <si>
+    <t>- All fields for Impact Outlook and Management Recommendation must be completed.</t>
+  </si>
+  <si>
+    <r>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>x.</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Do not leave any cell blank.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -363,8 +907,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,6 +955,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -420,116 +986,151 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="6">
+    <cellStyle name="20% - Accent6 2" xfId="5" xr:uid="{D7B5022D-E492-4FB7-B5D1-DE4067E2D67D}"/>
     <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
     <cellStyle name="40% - Accent2" xfId="2" builtinId="35"/>
     <cellStyle name="40% - Accent3" xfId="3" builtinId="39"/>
@@ -868,14 +1469,14 @@
       <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33" t="s">
+      <c r="E1" s="35"/>
+      <c r="F1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="33"/>
+      <c r="G1" s="35"/>
       <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -897,10 +1498,10 @@
       <c r="I2" s="27"/>
     </row>
     <row r="3" spans="1:9" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="34" t="s">
         <v>71</v>
       </c>
       <c r="C3" s="29" t="s">
@@ -948,7 +1549,7 @@
       <c r="A6" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="34" t="s">
         <v>72</v>
       </c>
       <c r="C6" s="29" t="s">
@@ -2455,14 +3056,14 @@
       <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33" t="s">
+      <c r="E1" s="35"/>
+      <c r="F1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="33"/>
+      <c r="G1" s="35"/>
       <c r="H1" s="11"/>
       <c r="I1" s="14"/>
     </row>
@@ -3684,15 +4285,443 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781F9F8-E2B4-4602-B993-31C422E594EE}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4634BE9-920B-457B-AEAD-CBA8166DFF39}">
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.5" customWidth="1"/>
+    <col min="2" max="6" width="19.125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+    </row>
+    <row r="2" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+      <c r="L2" s="41"/>
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B3" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42"/>
+    </row>
+    <row r="4" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="43" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B5" s="42" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B6" s="44" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="40"/>
+      <c r="C9" s="40"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="40"/>
+      <c r="F9" s="40"/>
+      <c r="G9" s="40"/>
+      <c r="H9" s="40"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B10" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B11" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="42"/>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B12" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B16" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="42"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="42"/>
+      <c r="F16" s="42"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="42"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="44" t="s">
+        <v>107</v>
+      </c>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="44"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="40"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="40" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="40"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="40"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="44" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="44"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B39" s="45"/>
+      <c r="C39" s="45"/>
+      <c r="D39" s="45"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="45"/>
+      <c r="G39" s="45"/>
+      <c r="H39" s="45"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="42" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="42"/>
+      <c r="D40" s="42"/>
+      <c r="E40" s="42"/>
+      <c r="F40" s="42"/>
+      <c r="G40" s="42"/>
+      <c r="H40" s="42"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="C41" s="44"/>
+      <c r="D41" s="44"/>
+      <c r="E41" s="44"/>
+      <c r="F41" s="44"/>
+      <c r="G41" s="44"/>
+      <c r="H41" s="44"/>
+    </row>
+    <row r="42" spans="1:8" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="45" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="B41:H41"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B6:H6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0780CF76-3B79-4709-9DEB-342DD9F5243B}">
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.125" customWidth="1"/>
+    <col min="2" max="2" width="86.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="46" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+    </row>
+    <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:2" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="38"/>
+    </row>
+    <row r="10" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="33" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="38"/>
+    </row>
+    <row r="16" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="73.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A15:B15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B020F0C-4030-5B4A-A41A-388920D315A9}">
   <dimension ref="A1:G83"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -3708,14 +4737,14 @@
       <c r="A1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34" t="s">
+      <c r="C1" s="36"/>
+      <c r="D1" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="34"/>
+      <c r="E1" s="36"/>
       <c r="F1" s="11"/>
       <c r="G1" s="14"/>
     </row>
@@ -4521,7 +5550,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D34D3AE-F2E2-3348-B195-43FB4D0F780C}">
   <dimension ref="A1:B40"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -4733,7 +5762,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B4F791-8893-1849-9452-A54B8C2F2F8E}">
   <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -4749,14 +5778,14 @@
       <c r="A1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35" t="s">
+      <c r="C1" s="37"/>
+      <c r="D1" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="35"/>
+      <c r="E1" s="37"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="20"/>
@@ -4954,7 +5983,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51686372-B2DE-1B43-8972-F1AC9C8B5F60}">
   <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Update durian and vegetable recommendations Excel files with new data.
</commit_message>
<xml_diff>
--- a/files/durian-recommendations.xlsx
+++ b/files/durian-recommendations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jusep\Desktop\PROJECTS\amia-microsite.github.io\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E8CFF1-42DE-4E24-AEB7-6744F25B73E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C987FA-29B2-4A9E-B781-7ABD9E9FD5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{E2D1DC89-D079-3B4D-864B-8CE149E3E279}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{E2D1DC89-D079-3B4D-864B-8CE149E3E279}"/>
   </bookViews>
   <sheets>
     <sheet name="Durian_10Day(Municipal)" sheetId="9" r:id="rId1"/>
@@ -754,6 +754,28 @@
     <t>6. Include crop insurance (PCIC) recommendations where appropriate, particularly during vulnerable crop stages such as flowering or fruiting.</t>
   </si>
   <si>
+    <t>- All fields for Impact Outlook and Management Recommendation must be completed.</t>
+  </si>
+  <si>
+    <r>
+      <t>e</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>x.</t>
+    </r>
+  </si>
+  <si>
+    <t>2. Do not leave any cell blank.</t>
+  </si>
+  <si>
     <r>
       <t>e</t>
     </r>
@@ -776,30 +798,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Recommend PCIC crop insurance enrollment during reproductive and maturing stages for high-value crops.</t>
+      <t xml:space="preserve"> Apply for PCIC crop insurance before planting and within 20 days after planting</t>
     </r>
-  </si>
-  <si>
-    <t>- All fields for Impact Outlook and Management Recommendation must be completed.</t>
-  </si>
-  <si>
-    <r>
-      <t>e</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>x.</t>
-    </r>
-  </si>
-  <si>
-    <t>2. Do not leave any cell blank.</t>
   </si>
 </sst>
 </file>
@@ -1092,18 +1092,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1113,11 +1101,14 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1125,8 +1116,17 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="5" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1469,14 +1469,14 @@
       <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35" t="s">
+      <c r="E1" s="40"/>
+      <c r="F1" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="35"/>
+      <c r="G1" s="40"/>
       <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -3056,14 +3056,14 @@
       <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35" t="s">
+      <c r="E1" s="40"/>
+      <c r="F1" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="35"/>
+      <c r="G1" s="40"/>
       <c r="H1" s="11"/>
       <c r="I1" s="14"/>
     </row>
@@ -4294,247 +4294,248 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
-      <c r="Q1" s="39"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
     </row>
     <row r="2" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="J2" s="41"/>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="M2" s="41"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="Q2" s="41"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="43"/>
     </row>
     <row r="4" spans="1:17" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="44" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="43" t="s">
         <v>99</v>
       </c>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="44"/>
-      <c r="H6" s="44"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="40" t="s">
+      <c r="A9" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="42"/>
-      <c r="D10" s="42"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="42"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="44" t="s">
+      <c r="B12" s="41" t="s">
         <v>104</v>
       </c>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
-      <c r="H12" s="44"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A15" s="40" t="s">
+      <c r="A15" s="42" t="s">
         <v>105</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="43" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="42"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="42"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="44" t="s">
+      <c r="B17" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="41"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="41"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="42" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
+      <c r="B20" s="42"/>
+      <c r="C20" s="42"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="42"/>
+      <c r="F20" s="42"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="42"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="42" t="s">
         <v>109</v>
       </c>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="44" t="s">
+      <c r="B24" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="C24" s="41"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="41"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="41"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="36"/>
+      <c r="E39" s="36"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="36"/>
+      <c r="H39" s="36"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B40" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="44"/>
-      <c r="F24" s="44"/>
-      <c r="G24" s="44"/>
-      <c r="H24" s="44"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B39" s="45"/>
-      <c r="C39" s="45"/>
-      <c r="D39" s="45"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="45"/>
-      <c r="G39" s="45"/>
-      <c r="H39" s="45"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="42" t="s">
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="43"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B41" s="41" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="42"/>
-      <c r="D40" s="42"/>
-      <c r="E40" s="42"/>
-      <c r="F40" s="42"/>
-      <c r="G40" s="42"/>
-      <c r="H40" s="42"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="44" t="s">
+      <c r="C41" s="41"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="41"/>
+    </row>
+    <row r="42" spans="1:8" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="36" t="s">
         <v>112</v>
-      </c>
-      <c r="C41" s="44"/>
-      <c r="D41" s="44"/>
-      <c r="E41" s="44"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="44"/>
-    </row>
-    <row r="42" spans="1:8" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="45" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="B10:H10"/>
@@ -4542,12 +4543,11 @@
     <mergeCell ref="B12:H12"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="B16:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B40:H40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4563,10 +4563,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="38" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4610,10 +4610,10 @@
     </row>
     <row r="8" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:2" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="39" t="s">
         <v>79</v>
       </c>
-      <c r="B9" s="38"/>
+      <c r="B9" s="39"/>
     </row>
     <row r="10" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
@@ -4649,10 +4649,10 @@
     </row>
     <row r="14" spans="1:2" ht="36.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38" t="s">
+      <c r="A15" s="39" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="38"/>
+      <c r="B15" s="39"/>
     </row>
     <row r="16" spans="1:2" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
@@ -4737,14 +4737,14 @@
       <c r="A1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36" t="s">
+      <c r="C1" s="45"/>
+      <c r="D1" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="36"/>
+      <c r="E1" s="45"/>
       <c r="F1" s="11"/>
       <c r="G1" s="14"/>
     </row>
@@ -5778,14 +5778,14 @@
       <c r="A1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37" t="s">
+      <c r="C1" s="46"/>
+      <c r="D1" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="37"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="20"/>

</xml_diff>